<commit_message>
Fix et modif d'onglets
</commit_message>
<xml_diff>
--- a/assets/documents/tableau_synthese.xlsx
+++ b/assets/documents/tableau_synthese.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="_-* #,##0.00\ [$€-1]_-;\-* #,##0.00\ [$€-1]_-;_-* &quot;-&quot;??\ [$€-1]_-"/>
   </numFmts>
-  <fonts count="17">
+  <fonts count="18">
     <font>
       <name val="Arial"/>
       <sz val="10"/>
@@ -109,6 +109,11 @@
       <b val="1"/>
       <sz val="11"/>
     </font>
+    <font>
+      <name val="Arial"/>
+      <b val="1"/>
+      <sz val="20"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -675,7 +680,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="76">
+  <cellXfs count="78">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -882,6 +887,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="15" fillId="0" borderId="16" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="26" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1317,12 +1328,12 @@
           <t>Option :</t>
         </is>
       </c>
-      <c r="G4" s="17" t="inlineStr">
+      <c r="G4" s="76" t="inlineStr">
         <is>
           <t>☐ SISR</t>
         </is>
       </c>
-      <c r="H4" s="56" t="inlineStr">
+      <c r="H4" s="77" t="inlineStr">
         <is>
           <t>☑ SLAM</t>
         </is>
@@ -1577,7 +1588,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="39.95" customFormat="1" customHeight="1" s="2">
+    <row r="14" ht="90" customFormat="1" customHeight="1" s="2">
       <c r="A14" s="63" t="inlineStr">
         <is>
           <t>MCP-serveur - Serveur Model Context Protocol
@@ -1768,7 +1779,7 @@
       <c r="G21" s="54" t="n"/>
       <c r="H21" s="55" t="n"/>
     </row>
-    <row r="22" ht="39.95" customFormat="1" customHeight="1" s="2">
+    <row r="22" ht="90" customFormat="1" customHeight="1" s="2">
       <c r="A22" s="72" t="inlineStr">
         <is>
           <t>Fondation.io - Comparateur d'IA Automatisé (Testing_Claude_code)
@@ -1801,7 +1812,7 @@
       </c>
       <c r="H22" s="22" t="n"/>
     </row>
-    <row r="23" ht="39.95" customFormat="1" customHeight="1" s="2">
+    <row r="23" ht="90" customFormat="1" customHeight="1" s="2">
       <c r="A23" s="72" t="inlineStr">
         <is>
           <t>Fondation.io - Scanner de Flux RSS Intelligent (RSSScanner)
@@ -1877,7 +1888,7 @@
       <c r="G28" s="54" t="n"/>
       <c r="H28" s="55" t="n"/>
     </row>
-    <row r="29" ht="30" customFormat="1" customHeight="1" s="2">
+    <row r="29" ht="90" customFormat="1" customHeight="1" s="2">
       <c r="A29" s="72" t="inlineStr">
         <is>
           <t>Fondation.io - AgentSea
@@ -2000,7 +2011,7 @@
     <mergeCell ref="A3:E3"/>
   </mergeCells>
   <printOptions horizontalCentered="1" verticalCentered="1"/>
-  <pageMargins left="0.1968503937007874" right="0.1968503937007874" top="0.1968503937007874" bottom="0.1968503937007874" header="0.5118110236220472" footer="0.5118110236220472"/>
-  <pageSetup orientation="portrait" paperSize="9" scale="48"/>
+  <pageMargins left="0.3" right="0.3" top="0.4" bottom="0.4" header="0.2" footer="0.2"/>
+  <pageSetup orientation="portrait" paperSize="9" fitToHeight="2" fitToWidth="1"/>
 </worksheet>
 </file>
</xml_diff>